<commit_message>
Document of Test plan and Verification plan
</commit_message>
<xml_diff>
--- a/Docs/AHB_test_plan.xlsx
+++ b/Docs/AHB_test_plan.xlsx
@@ -8,7 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Test Plan" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Coverage Plan" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="174">
   <si>
     <t xml:space="preserve">Test Plan</t>
   </si>
@@ -121,6 +122,9 @@
     <t xml:space="preserve">To ensure successful completion of multiple read transactions and verify the correctness of read data and AHB slave responses as per the protocol.</t>
   </si>
   <si>
+    <t xml:space="preserve">ahb_wr (HWRITE = 0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">back to back write</t>
   </si>
   <si>
@@ -143,6 +147,9 @@
   </si>
   <si>
     <t xml:space="preserve">To ensure continuous read transactions complete successfully with correct address sequencing, read data, and slave responses as per the AHB protocol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ahb_wr_wr (HWRITE=0)</t>
   </si>
   <si>
     <t xml:space="preserve">back to back write single 
@@ -464,7 +471,79 @@
     <t xml:space="preserve">make sim child=ahb_wr_rd_diff_size WAVE=1</t>
   </si>
   <si>
-    <t xml:space="preserve">  </t>
+    <t xml:space="preserve">change_addr_wait_state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address stability during wait state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes HADDR during an active wait state.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that the address remains stable while HREADY is LOW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remaining</t>
+  </si>
+  <si>
+    <t xml:space="preserve">change_hwrite_wait_state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hwrite stability during wait state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes HWRITE during an active wait state.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that the write control signal remains stable during wait states.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">change_hsize_wait_state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSIZE stability during wait state</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes HSIZE during an active wait state.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that the transfer size remains stable during wait states.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">change_transfer_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transfer type transitions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changes HTRANS between different transfer types.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify correct handling of IDLE, BUSY, NONSEQ and SEQ transfers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">addr_boundary_cross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Address boundary checking.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generates a burst transaction that attempts to cross a 1KB address boundary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that burst transfers do not cross the AHB 1KB boundary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">incorrect_burst_sequence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burst sequence validation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generates an invalid or unexpected burst transfer sequence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify that the DUT detects or handles incorrect burst sequences according to the protocol.</t>
   </si>
 </sst>
 </file>
@@ -558,7 +637,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -608,6 +687,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -734,7 +817,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.53"/>
@@ -920,34 +1003,43 @@
       <c r="F7" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="H7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -955,19 +1047,28 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>15</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -975,28 +1076,28 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J10" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1004,28 +1105,28 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1033,28 +1134,28 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1062,28 +1163,28 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1091,28 +1192,28 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1120,28 +1221,28 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1149,28 +1250,28 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1178,28 +1279,28 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1207,28 +1308,28 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1236,28 +1337,28 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1265,28 +1366,28 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1294,28 +1395,28 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1323,28 +1424,28 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1352,28 +1453,28 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1381,28 +1482,28 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1410,28 +1511,28 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1439,28 +1540,28 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1468,28 +1569,28 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1497,28 +1598,28 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1526,28 +1627,28 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1555,28 +1656,28 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1584,28 +1685,28 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,28 +1714,28 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D32" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="E32" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>138</v>
-      </c>
       <c r="I32" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1642,41 +1743,163 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E33" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F33" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>143</v>
-      </c>
       <c r="I33" s="2" t="s">
         <v>17</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="n">
         <v>31</v>
       </c>
+      <c r="B34" s="2" t="s">
+        <v>149</v>
+      </c>
       <c r="C34" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>150</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
         <v>32</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D35" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="n">
+        <v>33</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D36" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="n">
+        <v>34</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="D37" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="E37" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="n">
+        <v>35</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D38" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="D39" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="n">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1691,4 +1914,22 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>